<commit_message>
Update app with images and fixed nan values
</commit_message>
<xml_diff>
--- a/Fake_Calculator_2026.xlsx
+++ b/Fake_Calculator_2026.xlsx
@@ -615,7 +615,7 @@
         <v>30825000</v>
       </c>
       <c r="J2" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
@@ -725,7 +725,7 @@
         <v>30825000</v>
       </c>
       <c r="J3" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
@@ -835,7 +835,7 @@
         <v>30825000</v>
       </c>
       <c r="J4" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr">
@@ -945,7 +945,7 @@
         <v>30825000</v>
       </c>
       <c r="J5" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
@@ -1055,7 +1055,7 @@
         <v>30825000</v>
       </c>
       <c r="J6" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr">
@@ -1165,7 +1165,7 @@
         <v>30825000</v>
       </c>
       <c r="J7" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr">
@@ -1275,7 +1275,7 @@
         <v>30825000</v>
       </c>
       <c r="J8" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr">
@@ -1385,7 +1385,7 @@
         <v>30825000</v>
       </c>
       <c r="J9" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr">
@@ -1495,7 +1495,7 @@
         <v>30825000</v>
       </c>
       <c r="J10" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr">
@@ -1605,7 +1605,7 @@
         <v>30825000</v>
       </c>
       <c r="J11" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr">
@@ -1715,7 +1715,7 @@
         <v>30825000</v>
       </c>
       <c r="J12" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr">
@@ -1825,7 +1825,7 @@
         <v>30825000</v>
       </c>
       <c r="J13" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr">
@@ -1935,7 +1935,7 @@
         <v>30825000</v>
       </c>
       <c r="J14" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr">
@@ -2045,7 +2045,7 @@
         <v>30825000</v>
       </c>
       <c r="J15" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr">
@@ -2155,7 +2155,7 @@
         <v>30825000</v>
       </c>
       <c r="J16" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr">
@@ -2265,7 +2265,7 @@
         <v>30825000</v>
       </c>
       <c r="J17" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
@@ -2375,7 +2375,7 @@
         <v>30825000</v>
       </c>
       <c r="J18" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr">
@@ -2485,7 +2485,7 @@
         <v>30825000</v>
       </c>
       <c r="J19" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr">
@@ -2595,7 +2595,7 @@
         <v>30825000</v>
       </c>
       <c r="J20" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr">
@@ -2705,7 +2705,7 @@
         <v>30825000</v>
       </c>
       <c r="J21" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr">
@@ -7215,7 +7215,7 @@
         <v>30825000</v>
       </c>
       <c r="J62" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr">
@@ -7325,7 +7325,7 @@
         <v>30825000</v>
       </c>
       <c r="J63" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K63" t="inlineStr"/>
       <c r="L63" t="inlineStr">
@@ -7435,7 +7435,7 @@
         <v>30825000</v>
       </c>
       <c r="J64" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K64" t="inlineStr"/>
       <c r="L64" t="inlineStr">
@@ -7545,7 +7545,7 @@
         <v>30825000</v>
       </c>
       <c r="J65" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K65" t="inlineStr"/>
       <c r="L65" t="inlineStr">
@@ -7655,7 +7655,7 @@
         <v>30825000</v>
       </c>
       <c r="J66" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K66" t="inlineStr"/>
       <c r="L66" t="inlineStr">
@@ -7765,7 +7765,7 @@
         <v>30825000</v>
       </c>
       <c r="J67" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
@@ -7875,7 +7875,7 @@
         <v>30825000</v>
       </c>
       <c r="J68" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K68" t="inlineStr"/>
       <c r="L68" t="inlineStr">
@@ -7985,7 +7985,7 @@
         <v>30825000</v>
       </c>
       <c r="J69" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K69" t="inlineStr"/>
       <c r="L69" t="inlineStr">
@@ -8095,7 +8095,7 @@
         <v>30825000</v>
       </c>
       <c r="J70" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K70" t="inlineStr"/>
       <c r="L70" t="inlineStr">
@@ -8205,7 +8205,7 @@
         <v>30825000</v>
       </c>
       <c r="J71" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K71" t="inlineStr"/>
       <c r="L71" t="inlineStr">
@@ -8315,7 +8315,7 @@
         <v>30825000</v>
       </c>
       <c r="J72" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
@@ -8425,7 +8425,7 @@
         <v>30825000</v>
       </c>
       <c r="J73" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K73" t="inlineStr"/>
       <c r="L73" t="inlineStr">
@@ -8535,7 +8535,7 @@
         <v>30825000</v>
       </c>
       <c r="J74" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K74" t="inlineStr"/>
       <c r="L74" t="inlineStr">
@@ -8645,7 +8645,7 @@
         <v>30825000</v>
       </c>
       <c r="J75" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K75" t="inlineStr"/>
       <c r="L75" t="inlineStr">
@@ -8755,7 +8755,7 @@
         <v>30825000</v>
       </c>
       <c r="J76" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
@@ -8865,7 +8865,7 @@
         <v>30825000</v>
       </c>
       <c r="J77" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
@@ -8975,7 +8975,7 @@
         <v>30825000</v>
       </c>
       <c r="J78" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
@@ -9085,7 +9085,7 @@
         <v>30825000</v>
       </c>
       <c r="J79" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
@@ -9195,7 +9195,7 @@
         <v>30825000</v>
       </c>
       <c r="J80" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
@@ -9305,7 +9305,7 @@
         <v>30825000</v>
       </c>
       <c r="J81" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
@@ -13815,7 +13815,7 @@
         <v>28359000</v>
       </c>
       <c r="J122" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
@@ -13925,7 +13925,7 @@
         <v>28359000</v>
       </c>
       <c r="J123" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K123" t="inlineStr"/>
       <c r="L123" t="inlineStr">
@@ -14035,7 +14035,7 @@
         <v>28359000</v>
       </c>
       <c r="J124" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K124" t="inlineStr"/>
       <c r="L124" t="inlineStr">
@@ -14145,7 +14145,7 @@
         <v>28359000</v>
       </c>
       <c r="J125" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K125" t="inlineStr"/>
       <c r="L125" t="inlineStr">
@@ -14255,7 +14255,7 @@
         <v>28359000</v>
       </c>
       <c r="J126" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K126" t="inlineStr"/>
       <c r="L126" t="inlineStr">
@@ -14365,7 +14365,7 @@
         <v>28359000</v>
       </c>
       <c r="J127" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K127" t="inlineStr"/>
       <c r="L127" t="inlineStr">
@@ -14475,7 +14475,7 @@
         <v>28359000</v>
       </c>
       <c r="J128" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K128" t="inlineStr"/>
       <c r="L128" t="inlineStr">
@@ -14585,7 +14585,7 @@
         <v>28359000</v>
       </c>
       <c r="J129" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K129" t="inlineStr"/>
       <c r="L129" t="inlineStr">
@@ -14695,7 +14695,7 @@
         <v>28359000</v>
       </c>
       <c r="J130" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K130" t="inlineStr"/>
       <c r="L130" t="inlineStr">
@@ -14805,7 +14805,7 @@
         <v>28359000</v>
       </c>
       <c r="J131" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
@@ -14915,7 +14915,7 @@
         <v>28359000</v>
       </c>
       <c r="J132" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K132" t="inlineStr"/>
       <c r="L132" t="inlineStr">
@@ -15025,7 +15025,7 @@
         <v>28359000</v>
       </c>
       <c r="J133" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K133" t="inlineStr"/>
       <c r="L133" t="inlineStr">
@@ -15135,7 +15135,7 @@
         <v>28359000</v>
       </c>
       <c r="J134" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K134" t="inlineStr"/>
       <c r="L134" t="inlineStr">
@@ -15245,7 +15245,7 @@
         <v>28359000</v>
       </c>
       <c r="J135" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K135" t="inlineStr"/>
       <c r="L135" t="inlineStr">
@@ -15355,7 +15355,7 @@
         <v>28359000</v>
       </c>
       <c r="J136" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K136" t="inlineStr"/>
       <c r="L136" t="inlineStr">
@@ -15465,7 +15465,7 @@
         <v>28359000</v>
       </c>
       <c r="J137" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
@@ -15575,7 +15575,7 @@
         <v>28359000</v>
       </c>
       <c r="J138" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K138" t="inlineStr"/>
       <c r="L138" t="inlineStr">
@@ -15685,7 +15685,7 @@
         <v>28359000</v>
       </c>
       <c r="J139" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K139" t="inlineStr"/>
       <c r="L139" t="inlineStr">
@@ -15795,7 +15795,7 @@
         <v>28359000</v>
       </c>
       <c r="J140" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K140" t="inlineStr"/>
       <c r="L140" t="inlineStr">
@@ -15905,7 +15905,7 @@
         <v>28359000</v>
       </c>
       <c r="J141" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K141" t="inlineStr"/>
       <c r="L141" t="inlineStr">
@@ -18212,10 +18212,10 @@
         </is>
       </c>
       <c r="I162" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J162" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K162" t="inlineStr"/>
       <c r="L162" t="inlineStr">
@@ -18322,10 +18322,10 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J163" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K163" t="inlineStr"/>
       <c r="L163" t="inlineStr">
@@ -18432,10 +18432,10 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J164" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K164" t="inlineStr"/>
       <c r="L164" t="inlineStr">
@@ -18542,10 +18542,10 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J165" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K165" t="inlineStr"/>
       <c r="L165" t="inlineStr">
@@ -18652,10 +18652,10 @@
         </is>
       </c>
       <c r="I166" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J166" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K166" t="inlineStr"/>
       <c r="L166" t="inlineStr">
@@ -18762,10 +18762,10 @@
         </is>
       </c>
       <c r="I167" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J167" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K167" t="inlineStr"/>
       <c r="L167" t="inlineStr">
@@ -18872,10 +18872,10 @@
         </is>
       </c>
       <c r="I168" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J168" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K168" t="inlineStr"/>
       <c r="L168" t="inlineStr">
@@ -18982,10 +18982,10 @@
         </is>
       </c>
       <c r="I169" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J169" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K169" t="inlineStr"/>
       <c r="L169" t="inlineStr">
@@ -19092,10 +19092,10 @@
         </is>
       </c>
       <c r="I170" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J170" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K170" t="inlineStr"/>
       <c r="L170" t="inlineStr">
@@ -19202,10 +19202,10 @@
         </is>
       </c>
       <c r="I171" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J171" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K171" t="inlineStr"/>
       <c r="L171" t="inlineStr">
@@ -19312,10 +19312,10 @@
         </is>
       </c>
       <c r="I172" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J172" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K172" t="inlineStr"/>
       <c r="L172" t="inlineStr">
@@ -19422,10 +19422,10 @@
         </is>
       </c>
       <c r="I173" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J173" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K173" t="inlineStr"/>
       <c r="L173" t="inlineStr">
@@ -19532,10 +19532,10 @@
         </is>
       </c>
       <c r="I174" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J174" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K174" t="inlineStr"/>
       <c r="L174" t="inlineStr">
@@ -19642,10 +19642,10 @@
         </is>
       </c>
       <c r="I175" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J175" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K175" t="inlineStr"/>
       <c r="L175" t="inlineStr">
@@ -19752,10 +19752,10 @@
         </is>
       </c>
       <c r="I176" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J176" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K176" t="inlineStr"/>
       <c r="L176" t="inlineStr">
@@ -19862,10 +19862,10 @@
         </is>
       </c>
       <c r="I177" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J177" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K177" t="inlineStr"/>
       <c r="L177" t="inlineStr">
@@ -19972,10 +19972,10 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J178" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K178" t="inlineStr"/>
       <c r="L178" t="inlineStr">
@@ -20082,10 +20082,10 @@
         </is>
       </c>
       <c r="I179" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J179" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K179" t="inlineStr"/>
       <c r="L179" t="inlineStr">
@@ -20192,10 +20192,10 @@
         </is>
       </c>
       <c r="I180" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J180" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K180" t="inlineStr"/>
       <c r="L180" t="inlineStr">
@@ -20302,10 +20302,10 @@
         </is>
       </c>
       <c r="I181" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J181" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K181" t="inlineStr"/>
       <c r="L181" t="inlineStr">
@@ -20415,7 +20415,7 @@
         <v>28359000</v>
       </c>
       <c r="J182" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K182" t="inlineStr"/>
       <c r="L182" t="inlineStr">
@@ -20525,7 +20525,7 @@
         <v>28359000</v>
       </c>
       <c r="J183" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K183" t="inlineStr"/>
       <c r="L183" t="inlineStr">
@@ -20635,7 +20635,7 @@
         <v>28359000</v>
       </c>
       <c r="J184" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K184" t="inlineStr"/>
       <c r="L184" t="inlineStr">
@@ -20745,7 +20745,7 @@
         <v>28359000</v>
       </c>
       <c r="J185" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K185" t="inlineStr"/>
       <c r="L185" t="inlineStr">
@@ -20855,7 +20855,7 @@
         <v>28359000</v>
       </c>
       <c r="J186" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K186" t="inlineStr"/>
       <c r="L186" t="inlineStr">
@@ -20965,7 +20965,7 @@
         <v>28359000</v>
       </c>
       <c r="J187" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K187" t="inlineStr"/>
       <c r="L187" t="inlineStr">
@@ -21075,7 +21075,7 @@
         <v>28359000</v>
       </c>
       <c r="J188" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K188" t="inlineStr"/>
       <c r="L188" t="inlineStr">
@@ -21185,7 +21185,7 @@
         <v>28359000</v>
       </c>
       <c r="J189" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K189" t="inlineStr"/>
       <c r="L189" t="inlineStr">
@@ -21295,7 +21295,7 @@
         <v>28359000</v>
       </c>
       <c r="J190" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K190" t="inlineStr"/>
       <c r="L190" t="inlineStr">
@@ -21405,7 +21405,7 @@
         <v>28359000</v>
       </c>
       <c r="J191" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K191" t="inlineStr"/>
       <c r="L191" t="inlineStr">
@@ -21515,7 +21515,7 @@
         <v>28359000</v>
       </c>
       <c r="J192" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K192" t="inlineStr"/>
       <c r="L192" t="inlineStr">
@@ -21625,7 +21625,7 @@
         <v>28359000</v>
       </c>
       <c r="J193" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K193" t="inlineStr"/>
       <c r="L193" t="inlineStr">
@@ -21735,7 +21735,7 @@
         <v>28359000</v>
       </c>
       <c r="J194" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K194" t="inlineStr"/>
       <c r="L194" t="inlineStr">
@@ -21845,7 +21845,7 @@
         <v>28359000</v>
       </c>
       <c r="J195" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K195" t="inlineStr"/>
       <c r="L195" t="inlineStr">
@@ -21955,7 +21955,7 @@
         <v>28359000</v>
       </c>
       <c r="J196" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K196" t="inlineStr"/>
       <c r="L196" t="inlineStr">
@@ -22065,7 +22065,7 @@
         <v>28359000</v>
       </c>
       <c r="J197" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K197" t="inlineStr"/>
       <c r="L197" t="inlineStr">
@@ -22175,7 +22175,7 @@
         <v>28359000</v>
       </c>
       <c r="J198" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K198" t="inlineStr"/>
       <c r="L198" t="inlineStr">
@@ -22285,7 +22285,7 @@
         <v>28359000</v>
       </c>
       <c r="J199" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K199" t="inlineStr"/>
       <c r="L199" t="inlineStr">
@@ -22395,7 +22395,7 @@
         <v>28359000</v>
       </c>
       <c r="J200" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K200" t="inlineStr"/>
       <c r="L200" t="inlineStr">
@@ -22505,7 +22505,7 @@
         <v>28359000</v>
       </c>
       <c r="J201" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K201" t="inlineStr"/>
       <c r="L201" t="inlineStr">
@@ -24812,10 +24812,10 @@
         </is>
       </c>
       <c r="I222" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J222" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K222" t="inlineStr"/>
       <c r="L222" t="inlineStr">
@@ -24922,10 +24922,10 @@
         </is>
       </c>
       <c r="I223" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J223" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K223" t="inlineStr"/>
       <c r="L223" t="inlineStr">
@@ -25032,10 +25032,10 @@
         </is>
       </c>
       <c r="I224" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J224" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K224" t="inlineStr"/>
       <c r="L224" t="inlineStr">
@@ -25142,10 +25142,10 @@
         </is>
       </c>
       <c r="I225" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J225" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K225" t="inlineStr"/>
       <c r="L225" t="inlineStr">
@@ -25252,10 +25252,10 @@
         </is>
       </c>
       <c r="I226" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J226" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K226" t="inlineStr"/>
       <c r="L226" t="inlineStr">
@@ -25362,10 +25362,10 @@
         </is>
       </c>
       <c r="I227" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J227" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K227" t="inlineStr"/>
       <c r="L227" t="inlineStr">
@@ -25472,10 +25472,10 @@
         </is>
       </c>
       <c r="I228" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J228" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K228" t="inlineStr"/>
       <c r="L228" t="inlineStr">
@@ -25582,10 +25582,10 @@
         </is>
       </c>
       <c r="I229" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J229" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K229" t="inlineStr"/>
       <c r="L229" t="inlineStr">
@@ -25692,10 +25692,10 @@
         </is>
       </c>
       <c r="I230" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J230" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K230" t="inlineStr"/>
       <c r="L230" t="inlineStr">
@@ -25802,10 +25802,10 @@
         </is>
       </c>
       <c r="I231" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J231" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K231" t="inlineStr"/>
       <c r="L231" t="inlineStr">
@@ -25912,10 +25912,10 @@
         </is>
       </c>
       <c r="I232" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J232" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K232" t="inlineStr"/>
       <c r="L232" t="inlineStr">
@@ -26022,10 +26022,10 @@
         </is>
       </c>
       <c r="I233" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J233" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K233" t="inlineStr"/>
       <c r="L233" t="inlineStr">
@@ -26132,10 +26132,10 @@
         </is>
       </c>
       <c r="I234" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J234" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K234" t="inlineStr"/>
       <c r="L234" t="inlineStr">
@@ -26242,10 +26242,10 @@
         </is>
       </c>
       <c r="I235" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J235" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K235" t="inlineStr"/>
       <c r="L235" t="inlineStr">
@@ -26352,10 +26352,10 @@
         </is>
       </c>
       <c r="I236" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J236" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K236" t="inlineStr"/>
       <c r="L236" t="inlineStr">
@@ -26462,10 +26462,10 @@
         </is>
       </c>
       <c r="I237" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J237" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K237" t="inlineStr"/>
       <c r="L237" t="inlineStr">
@@ -26572,10 +26572,10 @@
         </is>
       </c>
       <c r="I238" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J238" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K238" t="inlineStr"/>
       <c r="L238" t="inlineStr">
@@ -26682,10 +26682,10 @@
         </is>
       </c>
       <c r="I239" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J239" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K239" t="inlineStr"/>
       <c r="L239" t="inlineStr">
@@ -26792,10 +26792,10 @@
         </is>
       </c>
       <c r="I240" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J240" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K240" t="inlineStr"/>
       <c r="L240" t="inlineStr">
@@ -26902,10 +26902,10 @@
         </is>
       </c>
       <c r="I241" t="n">
-        <v>8220000.000000001</v>
+        <v>8220000</v>
       </c>
       <c r="J241" t="n">
-        <v>7924080.000000001</v>
+        <v>7924080</v>
       </c>
       <c r="K241" t="inlineStr"/>
       <c r="L241" t="inlineStr">
@@ -40215,7 +40215,7 @@
         <v>30825000</v>
       </c>
       <c r="J362" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K362" t="inlineStr"/>
       <c r="L362" t="inlineStr">
@@ -40325,7 +40325,7 @@
         <v>30825000</v>
       </c>
       <c r="J363" t="n">
-        <v>29484112.5</v>
+        <v>29484113</v>
       </c>
       <c r="K363" t="inlineStr"/>
       <c r="L363" t="inlineStr">
@@ -40435,7 +40435,7 @@
         <v>28359000</v>
       </c>
       <c r="J364" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K364" t="inlineStr"/>
       <c r="L364" t="inlineStr">
@@ -40545,7 +40545,7 @@
         <v>28359000</v>
       </c>
       <c r="J365" t="n">
-        <v>27125383.5</v>
+        <v>27125384</v>
       </c>
       <c r="K365" t="inlineStr"/>
       <c r="L365" t="inlineStr">

</xml_diff>